<commit_message>
Updated ASR Intelligence Lab Pro with microphone, IndicWhisper and fixes
</commit_message>
<xml_diff>
--- a/asr_lab_pro_logs.xlsx
+++ b/asr_lab_pro_logs.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N64"/>
+  <dimension ref="A1:N69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3506,6 +3506,234 @@
         <v>1</v>
       </c>
     </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>Whisper</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>People are tough to feed. But the nation thinks that Iran can't be trusted unless they succeed.</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="D65" t="n">
+        <v>10.659</v>
+      </c>
+      <c r="E65" t="n">
+        <v>1.6951</v>
+      </c>
+      <c r="F65" t="inlineStr"/>
+      <c r="G65" t="inlineStr"/>
+      <c r="H65" t="inlineStr"/>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="J65" t="inlineStr"/>
+      <c r="K65" t="inlineStr">
+        <is>
+          <t>2026-07-01T13:14:53</t>
+        </is>
+      </c>
+      <c r="L65" t="n">
+        <v>6.288</v>
+      </c>
+      <c r="M65" t="inlineStr">
+        <is>
+          <t>🌐 Auto Detect</t>
+        </is>
+      </c>
+      <c r="N65" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>Faster-Whisper</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>இங்கள ஒரே பேசு செய்வேக்கு வரவே இருக்கிறாம். நான் உங்களையைக் குழல் புதவியாலே.</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>ta</t>
+        </is>
+      </c>
+      <c r="D66" t="n">
+        <v>2.17</v>
+      </c>
+      <c r="E66" t="n">
+        <v>0.3451</v>
+      </c>
+      <c r="F66" t="inlineStr"/>
+      <c r="G66" t="inlineStr"/>
+      <c r="H66" t="inlineStr"/>
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="J66" t="inlineStr"/>
+      <c r="K66" t="inlineStr">
+        <is>
+          <t>2026-07-01T13:14:53</t>
+        </is>
+      </c>
+      <c r="L66" t="n">
+        <v>6.288</v>
+      </c>
+      <c r="M66" t="inlineStr">
+        <is>
+          <t>🌐 Auto Detect</t>
+        </is>
+      </c>
+      <c r="N66" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>Sarvam AI</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr"/>
+      <c r="C67" t="inlineStr"/>
+      <c r="D67" t="n">
+        <v>0</v>
+      </c>
+      <c r="E67" t="n">
+        <v>0</v>
+      </c>
+      <c r="F67" t="inlineStr"/>
+      <c r="G67" t="inlineStr"/>
+      <c r="H67" t="inlineStr"/>
+      <c r="I67" t="inlineStr">
+        <is>
+          <t>skipped</t>
+        </is>
+      </c>
+      <c r="J67" t="inlineStr">
+        <is>
+          <t>No Sarvam API key</t>
+        </is>
+      </c>
+      <c r="K67" t="inlineStr">
+        <is>
+          <t>2026-07-01T13:14:53</t>
+        </is>
+      </c>
+      <c r="L67" t="n">
+        <v>6.288</v>
+      </c>
+      <c r="M67" t="inlineStr">
+        <is>
+          <t>🌐 Auto Detect</t>
+        </is>
+      </c>
+      <c r="N67" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>Shrutam</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr"/>
+      <c r="C68" t="inlineStr"/>
+      <c r="D68" t="n">
+        <v>0</v>
+      </c>
+      <c r="E68" t="n">
+        <v>0</v>
+      </c>
+      <c r="F68" t="inlineStr"/>
+      <c r="G68" t="inlineStr"/>
+      <c r="H68" t="inlineStr"/>
+      <c r="I68" t="inlineStr">
+        <is>
+          <t>skipped</t>
+        </is>
+      </c>
+      <c r="J68" t="inlineStr">
+        <is>
+          <t>IndicWhisper safe mode: transformers not installed</t>
+        </is>
+      </c>
+      <c r="K68" t="inlineStr">
+        <is>
+          <t>2026-07-01T13:14:53</t>
+        </is>
+      </c>
+      <c r="L68" t="n">
+        <v>6.288</v>
+      </c>
+      <c r="M68" t="inlineStr">
+        <is>
+          <t>🌐 Auto Detect</t>
+        </is>
+      </c>
+      <c r="N68" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>Gemini</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr"/>
+      <c r="C69" t="inlineStr"/>
+      <c r="D69" t="n">
+        <v>0</v>
+      </c>
+      <c r="E69" t="n">
+        <v>0</v>
+      </c>
+      <c r="F69" t="inlineStr"/>
+      <c r="G69" t="inlineStr"/>
+      <c r="H69" t="inlineStr"/>
+      <c r="I69" t="inlineStr">
+        <is>
+          <t>skipped</t>
+        </is>
+      </c>
+      <c r="J69" t="inlineStr">
+        <is>
+          <t>Safe mode: no Gemini API key</t>
+        </is>
+      </c>
+      <c r="K69" t="inlineStr">
+        <is>
+          <t>2026-07-01T13:14:53</t>
+        </is>
+      </c>
+      <c r="L69" t="n">
+        <v>6.288</v>
+      </c>
+      <c r="M69" t="inlineStr">
+        <is>
+          <t>🌐 Auto Detect</t>
+        </is>
+      </c>
+      <c r="N69" t="b">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>